<commit_message>
Komisyon ücretleri güncellendi (31.07.2026)
</commit_message>
<xml_diff>
--- a/garanti_komisyonlar.xlsx
+++ b/garanti_komisyonlar.xlsx
@@ -492,19 +492,16 @@
           <t>0.27TL</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>0.27TL</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>BSMV hariç.Güncellenme Tarihi: 01.03.2020 00:00</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -560,19 +557,16 @@
           <t>39.87TL</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>797.68TL</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>BSMV Hariç. 0-8.300 TL arası 39,87 TL;8.300,01-399.000 TL arası 57,14 TL; 399.000 TL üzeri 797,68 TL masraflıdır.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -595,14 +589,11 @@
           <t>2.9%</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>BSMV Hariç. Oran limit üzeri çekilen tutara aittir. İşleme ilişkin ücret tutarı ve oran değişebilecektir. ATM’lerden yapılacak işlem anında müşteri bilgilendirmesi yapılarak onay alınır. Güncellenme Tarihi: 10.07.2026</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -625,14 +616,11 @@
           <t>2.9%</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>BSMV Hariç. Oran limit üzeri çekilen tutara aittir. İşleme ilişkin ücret tutarı ve oran değişebilecektir. ATM’lerden yapılacak işlem anında müşteri bilgilendirmesi yapılarak onay alınır. Güncellenme Tarihi: 10.07.2026</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -655,14 +643,11 @@
           <t>2.9%</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>BSMV Hariç. Oran limit üzeri çekilen tutara aittir. İşleme ilişkin ücret tutarı ve oran değişebilecektir. ATM’lerden yapılacak işlem anında müşteri bilgilendirmesi yapılarak onay alınır. Güncellenme Tarihi: 10.07.2026</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -685,14 +670,11 @@
           <t>2.9%</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>BSMV Hariç. Oran limit üzeri çekilen tutara aittir. İşleme ilişkin ücret tutarı ve oran değişebilecektir. ATM’lerden yapılacak işlem anında müşteri bilgilendirmesi yapılarak onay alınır. Güncellenme Tarihi: 10.07.2026</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -800,19 +782,16 @@
           <t>27.84TL</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>27.84TL</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>BSMV Hariç. Kredi Kartından yapılan EFT işlemlerinde EFT ücretine ek olarak %1 nakit avans ücreti ve nakit avans faizi uygulanmaktadır. Güncellenme Tarihi: 06.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -830,19 +809,16 @@
           <t>55.69TL</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>55.69TL</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>BSMV Hariç. Kredi Kartından yapılan EFT işlemlerinde EFT ücretine ek olarak %1 nakit avans ücreti ve nakit avans faizi uygulanmaktadır. Güncellenme Tarihi: 06.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -860,19 +836,16 @@
           <t>398.83TL</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>398.83TL</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>BSMV Hariç. Kredi Kartından yapılan EFT işlemlerinde EFT ücretine ek olarak %1 nakit avans ücreti ve nakit avans faizi uygulanmaktadır. Güncellenme Tarihi: 06.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -890,19 +863,16 @@
           <t>39.87TL</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>39.87TL</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>BSMV Hariç Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -920,19 +890,16 @@
           <t>79.76TL</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>79.76TL</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>BSMV Hariç Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -950,19 +917,16 @@
           <t>797.68TL</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>797.68TL</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>BSMV Hariç Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1100,19 +1064,16 @@
           <t>27.85TL</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>27.85TL</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>BSMV Hariç. Kredi Kartından yapılan İşlemlerde EFT/Havale ücretine ek olarak %1 nakit avans ücreti ve nakit avans faizi uygulanmaktadır. Güncellenme Tarihi: 06.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1130,19 +1091,16 @@
           <t>199.42TL</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>199.42TL</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>BSMV Hariç. Kredi Kartından yapılan İşlemlerde EFT/Havale ücretine ek olarak %1 nakit avans ücreti ve nakit avans faizi uygulanmaktadır. Güncellenme Tarihi: 06.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1160,19 +1118,16 @@
           <t>19.94TL</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>19.94TL</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1190,19 +1145,16 @@
           <t>39.88TL</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>39.88TL</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1220,19 +1172,16 @@
           <t>398.84TL</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>398.84TL</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1270,7 +1219,6 @@
           <t>Garanti BBVA International'dan Gelen Havale. BSMV hariç.Güncellenme Tarihi: 05.02.2026 00:00</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1288,19 +1236,16 @@
           <t>15.00USD</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>220.00USD</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>BSMV Hariç.İnternetten yapılırsa asgari tutar 5 USD, azami tutar 80 USD. Güncellenme Tarihi: 01.03.2020 00:00</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1318,19 +1263,16 @@
           <t>190.48TL</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>190.48TL</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>BSMV Hariç. İşlem bazında ve mesajın çekildiği anda. Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1348,19 +1290,16 @@
           <t>309.52TL</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>309.52TL</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>BSMV Hariç. Güncellenme Tarihi:10.12.2025 00:00</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1398,7 +1337,6 @@
           <t>BSMV Hariç. Güncellenme Tarihi:10.12.2025 00:00</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1416,19 +1354,16 @@
           <t>171.43TL</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>171.43TL</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>BSMV Hariç. Güncellenme Tarihi:10.12.2025 00:00</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1466,7 +1401,6 @@
           <t>BSMV Hariç. Güncellenme Tarihi:10.12.2025 00:00</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1504,7 +1438,6 @@
           <t>BSMV hariç.Güncellenme Tarihi: 05.02.2026 00:00</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1522,19 +1455,16 @@
           <t>1050.00TL</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>1050.00TL</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>BSMV dahil.Belirtilen ücretler para transferi komisyon ücreti olup, gönderim seçeneklerine bağlı olarak işleme aracılık eden bankalar tarafından muhabir bankası masrafı ayrıca tahsil edilebilecektir. Dolayısıyla Swift işlemlerinde alıcının eline geçen tutar gönderilen tutardan daha düşük olabilir.Güncellenme Tarihi: 05.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1552,19 +1482,16 @@
           <t>1250.00TL</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>1250.00TL</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>BSMV dahil.Belirtilen ücretler para transferi komisyon ücreti olup, gönderim seçeneklerine bağlı olarak işleme aracılık eden bankalar tarafından muhabir bankası masrafı ayrıca tahsil edilebilecektir. Dolayısıyla Swift işlemlerinde alıcının eline geçen tutar gönderilen tutardan daha düşük olabilir.Güncellenme Tarihi: 05.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1582,19 +1509,16 @@
           <t>1500.00TL</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>1500.00TL</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>BSMV dahil.Belirtilen ücretler para transferi komisyon ücreti olup, gönderim seçeneklerine bağlı olarak işleme aracılık eden bankalar tarafından muhabir bankası masrafı ayrıca tahsil edilebilecektir. Dolayısıyla Swift işlemlerinde alıcının eline geçen tutar gönderilen tutardan daha düşük olabilir.Güncellenme Tarihi: 05.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1632,7 +1556,6 @@
           <t>BSMV dahil.Belirtilen ücretler para transferi komisyon ücreti olup, gönderim seçeneklerine bağlı olarak işleme aracılık eden bankalar tarafından muhabir bankası masrafı ayrıca tahsil edilebilecektir. Dolayısıyla Swift işlemlerinde alıcının eline geçen tutar gönderilen tutardan daha düşük olabilir.Güncellenme Tarihi: 05.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1650,19 +1573,16 @@
           <t>2485.72TL</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>2485.72TL</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>BSMV hariç.Belirtilen ücretler para transferi komisyon ücreti olup, gönderim seçeneklerine bağlı olarak işleme aracılık eden bankalar tarafından muhabir bankası masrafı ayrıca tahsil edilebilecektir. Dolayısıyla Swift işlemlerinde alıcının eline geçen tutar gönderilen tutardan daha düşük olabilir.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1680,19 +1600,16 @@
           <t>2733.34TL</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>2733.34TL</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>BSMV hariç.Belirtilen ücretler para transferi komisyon ücreti olup, gönderim seçeneklerine bağlı olarak işleme aracılık eden bankalar tarafından muhabir bankası masrafı ayrıca tahsil edilebilecektir. Dolayısıyla Swift işlemlerinde alıcının eline geçen tutar gönderilen tutardan daha düşük olabilir.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1710,19 +1627,16 @@
           <t>2923.81TL</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>2923.81TL</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>BSMV hariç.Belirtilen ücretler para transferi komisyon ücreti olup, gönderim seçeneklerine bağlı olarak işleme aracılık eden bankalar tarafından muhabir bankası masrafı ayrıca tahsil edilebilecektir. Dolayısıyla Swift işlemlerinde alıcının eline geçen tutar gönderilen tutardan daha düşük olabilir.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1760,7 +1674,6 @@
           <t>BSMV hariç.Belirtilen ücretler para transferi komisyon ücreti olup, gönderim seçeneklerine bağlı olarak işleme aracılık eden bankalar tarafından muhabir bankası masrafı ayrıca tahsil edilebilecektir. Dolayısıyla Swift işlemlerinde alıcının eline geçen tutar gönderilen tutardan daha düşük olabilir.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1778,19 +1691,16 @@
           <t>50.00TL</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>50.00TL</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 01.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1808,19 +1718,16 @@
           <t>100.00TL</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>100.00TL</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 01.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1838,19 +1745,16 @@
           <t>7.97TL</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>7.97TL</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>BSMV Hariç. Güncellenme Tarihi: 06.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1868,19 +1772,16 @@
           <t>15.96TL</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>15.96TL</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>BSMV Hariç. Güncellenme Tarihi: 06.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1898,19 +1799,16 @@
           <t>30000.00TL</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>30000.00TL</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>BSMV dahildir. Söz konusu ücretler 18.05.2026 tarihi itibarıyla yeni açılan kiralık kasalar için geçerli fiyatlardır. Bu tarihten önce açılan kiralık kasalar ücretler bakımından farklılık gösterebilecektir. Söz konusu ücretlerde değişiklik yapılması halinde gerekli bilgilendirme yapılacaktır.</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1928,19 +1826,16 @@
           <t>22000.00TL</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>22000.00TL</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>BSMV dahildir. Söz konusu ücretler 18.05.2026 tarihi itibarıyla yeni açılan kiralık kasalar için geçerli fiyatlardır. Bu tarihten önce açılan kiralık kasalar ücretler bakımından farklılık gösterebilecektir. Söz konusu ücretlerde değişiklik yapılması halinde gerekli bilgilendirme yapılacaktır.</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1958,19 +1853,16 @@
           <t>25000.00TL</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
           <t>25000.00TL</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>BSMV dahildir. Söz konusu ücretler 18.05.2026 tarihi itibarıyla yeni açılan kiralık kasalar için geçerli fiyatlardır. Bu tarihten önce açılan kiralık kasalar ücretler bakımından farklılık gösterebilecektir. Söz konusu ücretlerde değişiklik yapılması halinde gerekli bilgilendirme yapılacaktır.</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -1988,19 +1880,16 @@
           <t>28570.00TL</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
           <t>28570.00TL</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>BSMV hariçtir.* Söz konusu ücretler 18.05.2026 tarihi itibarıyla yeni açılan kiralık kasalar için geçerli fiyatlardır. Bu tarihten önce açılan kiralık kasalar ücretler bakımından farklılık gösterebilecektir. Söz konusu ücretlerde değişiklik yapılması halinde gerekli bilgilendirme yapılacaktır.</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2018,19 +1907,16 @@
           <t>23805.00TL</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>23805.00TL</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>BSMV hariçtir.* Söz konusu ücretler 18.05.2026 tarihi itibarıyla yeni açılan kiralık kasalar için geçerli fiyatlardır. Bu tarihten önce açılan kiralık kasalar ücretler bakımından farklılık gösterebilecektir. Söz konusu ücretlerde değişiklik yapılması halinde gerekli bilgilendirme yapılacaktır.</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2048,19 +1934,16 @@
           <t>20950.00TL</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>20950.00TL</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>BSMV hariçtir.* Söz konusu ücretler 18.05.2026 tarihi itibarıyla yeni açılan kiralık kasalar için geçerli fiyatlardır. Bu tarihten önce açılan kiralık kasalar ücretler bakımından farklılık gösterebilecektir. Söz konusu ücretlerde değişiklik yapılması halinde gerekli bilgilendirme yapılacaktır.</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2078,19 +1961,16 @@
           <t>287.62TL</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
           <t>287.62TL</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>Son 1 sene ücretsiz. 1 seneden eski- 3 seneden yeni tarihli dökümanlar 28.58 TL. 3 seneden eski tarihli dökümanlar 287.62 TL'dir.BSMV hariç.Güncellenme Tarihi: 05.02.2026 00:00</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2128,7 +2008,6 @@
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2146,19 +2025,16 @@
           <t>85.72TL</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
           <t>85.72TL</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>BSMV hariç. Değerli kağıt vergisi hariç. Tutar şube kanalına aittir. Dijitalden çek başvurusunda ücret 76,20 TL'dir. Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2176,19 +2052,16 @@
           <t>133.34TL</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>133.34TL</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2226,7 +2099,6 @@
           <t>BSMV Hariç.Güncellenme Tarihi: 01.04.2020 00:00</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2244,19 +2116,16 @@
           <t>114.29TL</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>114.29TL</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2274,19 +2143,16 @@
           <t>171.43TL</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>171.43TL</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2304,19 +2170,16 @@
           <t>438.10TL</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
           <t>438.10TL</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2334,19 +2197,16 @@
           <t>1469.52TL</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>1469.52TL</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 14.04.2026 00:00</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2384,7 +2244,6 @@
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2402,19 +2261,16 @@
           <t>323.81TL</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
           <t>323.81TL</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2432,7 +2288,6 @@
           <t>45.00USD</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
           <t>45.00USD</t>
@@ -2448,7 +2303,6 @@
           <t>BSMV Hariç. Muhabir borç geçtiğinde, muhabirin borç geçtiği tutar;İşlem bazında Ödeme anında (Yurtdışından Tahsile Gelen Çeklerin Ödenmesi (Normal YP Çek) Güncellenme Tarihi: 01.04.2021 00:00</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2466,19 +2320,16 @@
           <t>257.15TL</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
           <t>257.15TL</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2496,19 +2347,16 @@
           <t>390.48TL</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
           <t>390.48TL</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2556,19 +2404,16 @@
           <t>495.24TL</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
           <t>495.24TL</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2586,19 +2431,16 @@
           <t>533.34TL</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
           <t>533.34TL</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2616,19 +2458,16 @@
           <t>600.00TL</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
           <t>600.00TL</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2646,19 +2485,16 @@
           <t>600.00TL</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
           <t>600.00TL</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 09.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2676,19 +2512,16 @@
           <t>275.00TL</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
           <t>275.00TL</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>BSMV Dahil .Güncellenme Tarihi: 09.02.2026 17:35</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2706,19 +2539,16 @@
           <t>550.00TL</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
           <t>550.00TL</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>BSMV Dahil .Güncellenme Tarihi: 09.02.2026 17:35</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2736,19 +2566,16 @@
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 22.07.2026 00:00</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2766,19 +2593,16 @@
           <t>3.99TL</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
           <t>232.23TL</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>BSMV Hariç. Azami Tutar Satıcı Komisyonudur. Alıcı komisyonu min. 3,99 TL max 99,71 TL'dir. Güncellenme Tarihi: 06.01.2026</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2826,8 +2650,6 @@
           <t>5.00TL</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
           <t>3.50%</t>
@@ -2838,7 +2660,6 @@
           <t>Bu ücretler tahsilat sistemi anlaşması bulunan site vb. kurumlar için de geçerlidir. 149.99 TL’ye kadar olan ödemelerde asgâri tutar, 150.00 TL ve üzeri ödemelerde azami oran tahsil edilir. BSMV dahil.Güncellenme Tarihi: 25.07.2023</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2856,19 +2677,16 @@
           <t>30.00TL</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
           <t>36.00TL</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>BSMV Hariç. Bilyoner, Nesine, Tuttur, Oley, Misli, Sisal Şans, Birebin, TJK için tahsilat yapılmaktadır. Kanal bazında ücret farklılık göstermektedir. Güncellenme Tarihi: 01.01.2026 00:00</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2916,19 +2734,16 @@
           <t>15975.00TL</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
           <t>81665.00TL</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>Ekspertiz ücreti değerlemeye konu gayrimenkulün konumu, vasfı ve brüt alanına (m2) göre değişiklik göstermektedir. Ekspertiz hizmeti için oluşan ve üçüncü kişilere, kurum/kuruluşlara ödenen maliyet tutarı tahsil edilir. BSMV’den muaftır.</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2946,19 +2761,16 @@
           <t>17135.00TL</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
           <t>227785.00TL</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>Ekspertiz ücreti değerlemeye konu gayrimenkulün konumu, vasfı ve brüt alanına (m2) göre değişiklik göstermektedir. Ekspertiz hizmeti için oluşan ve üçüncü kişilere, kurum/kuruluşlara ödenen maliyet tutarı tahsil edilir. BSMV dahildir.</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -2976,15 +2788,11 @@
           <t>900.00TL</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>Sigorta tutarı yaşa ve teminata göre değişiklik gösterebilir.</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3002,19 +2810,16 @@
           <t>100.00TL</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
           <t>900.00TL</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>Sigorta tutarı yaşa ve teminata göre değişiklik gösterebilir.</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3032,8 +2837,6 @@
           <t>10000.00TL</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
-      <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
           <t>6.50%</t>
@@ -3044,7 +2847,6 @@
           <t>Yıllık max oranı geçmeyecek şekilde dönemsel olarak tahsil edilir. %6,5'in 10000 TL'den daha düşük olması halinde 10000 TL komisyon tahsil edilir. BSMV Hariç.</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3062,8 +2864,6 @@
           <t>10000.00TL</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
           <t>6.50%</t>
@@ -3074,7 +2874,6 @@
           <t>Yıllık max oranı geçmeyecek şekilde dönemsel olarak tahsil edilir. %6,5'in 10000 TL'den daha düşük olması halinde 10000 TL komisyon tahsil edilir. BSMV Hariç.</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3182,8 +2981,6 @@
           <t>45USD</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>0.15%</t>
@@ -3194,7 +2991,6 @@
           <t>İşlem bazında - Ödeme anında (Yurtdışından Tahsile Gelen Çeklerin Ödenmesi (normal YP Çek)</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3212,7 +3008,6 @@
           <t>40USD</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
           <t>240USD</t>
@@ -3228,7 +3023,6 @@
           <t>İşlem Bazında ve transfer aşamasında (İleri gün valörlü peşin ve mal mukabili ithalat ödemeleri)</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3246,19 +3040,16 @@
           <t>4000.00TL</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
           <t>4000.00TL</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>BSMV Hariç.Güncellenme Tarihi: 07.08.2025 00:00</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3276,8 +3067,6 @@
           <t>2600.00TL</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
-      <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr">
         <is>
           <t>15.00%</t>
@@ -3288,7 +3077,6 @@
           <t>BSMV hariç.</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3306,15 +3094,11 @@
           <t>1350.00</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>Sigorta tutarı yaşa ve teminata göre değişiklik gösterebilir.</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3332,15 +3116,11 @@
           <t>1350</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr"/>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>Sigorta tutarı yaşa ve teminata göre değişiklik gösterebilir.</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3358,19 +3138,16 @@
           <t>0.27TL</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
           <t>0.27TL</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>BSMV eklenir.</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3393,14 +3170,11 @@
           <t>1.15%</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>BSMV eklenir.</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3448,19 +3222,16 @@
           <t>99.00TL</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
           <t>2400.00TL</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>Asıl ve ek kartlarınızı, kayıp/çalıntı vb. nedenler ile 1 takvim yılı içinde 2 kez ücretsiz yenileyebilirsiniz. 3. yenilemeden itibaren ise her bir kart yenilemesinde;American Express Metal The Platinum Card için 2.400 TL, Bonus Platinum Biyometrik kart için 500 TL, diğer kartlar için 99 TL ücret yansıtılacaktır.</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3498,7 +3269,6 @@
           <t>0 -1,500 TL'ye %2.00+15 TL - 1,500 -5,000 TL'ye %2.00+30 TL - 5,000 TL üzerine %1.50+40 TL ücret alınır ve BSMV eklenir.</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3717,14 +3487,11 @@
           <t>1.00%</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr"/>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>Karttan Havale/EFT işlemlerinde işlem tutarı üzerinden %1 oranında nakit avans işlem ücreti uygulanır (BSMV Hariç). Buna ek olarak,Garanti BBVA Mobil ve İnternet Bankacılığı’ndan yapılan işlemlerde:EFT işlemleri için 0-8.300 TL arasına 7,97 TL, 8.300-399.000 TL arasına 15,96 TL, 399.000 TL üzerine ise 199,41 TL EFT ücreti, Havale işlemleri için 0-8.300 TL arasına 3,99 TL, 8.300-399.000 TL arasına 7,98 TL, 399.000 TL üzerine ise 99,71 TL havale ücreti alınacaktır (BSMV hariç).Garanti BBVA ATM’lerinden yapılan işlemlerde:EFT işlemleri için 0-8.300 TL arasına 27,84 TL, 8.300-399.000 TL arasına 55,69 TL, 399.000 TL üzerine ise 398,83 TL EFT ücreti, Havale işlemleri için 0-8.300 TL arasına 13,92 TL, 8.300-399.000 TL arasına 27,85 TL, 399.000 TL üzerine ise 199,42 TL havale ücreti alınacaktır (BSMV hariç).Ayrıca Karttan Havale/EFT kullanımlarında işlem tarihinden itibaren günlük nakit faizi işletilir.</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3742,19 +3509,16 @@
           <t>140.00TL</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
           <t>3000.00TL</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>Asıl ve ek kartlarınızı, kayıp/çalıntı vb. nedenler ile 1 takvim yılı içinde 2 kez ücretsiz yenileyebilirsiniz. 3. yenilemeden itibaren ise her bir kart yenilemesinde; American Express Metal The Platinum için 3.000 TL, Bonus Platinum Biyometrik için 1.547 TL, Bonus Platinum Dinamik için 1.066 TL, diger kartlar için 140 TL ücret yansıtılacaktır.</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3777,14 +3541,11 @@
           <t>3.50%</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>100 TL altı işlemler için Asgari Tutar , 100 TL ve üzerindeki işlemler için Asgari Oran uygulanır.</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3802,15 +3563,11 @@
           <t>0.00TL</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
           <t>0.00TL</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3828,19 +3585,16 @@
           <t>750.00TL</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
           <t>750.00TL</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>BSMV dahildir. 6 aylık dönemlerde, yılda iki kere tahsilat yapılmaktadır.Yabancı para cinsi vadesiz hesaplardan yapılacak tahsilatlarda 750 TL muadili ücret tahsilat anında; açıklanan en güncel merkez bankası döviz kuruna göre belirlenecektir</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3888,19 +3642,16 @@
           <t>0.45EUR</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr">
         <is>
           <t>0.45EUR</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>Muadili ücret tahsil edilmektedir. Talep edilen ekstre başına tahsilat yapılmaktadır. BSMV dahildir.</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3918,19 +3669,16 @@
           <t>250.00TL</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr">
         <is>
           <t>250.00TL</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
           <t>Hisse senedi hesaplarından 6 ayda bir 250 TL (BSMV dahil) (yıllık 500 TL (BSMV dahil)) hesap bakım ücreti tahsil edilmektedir. Yıllık hesap bakım ücreti hisse senedi satış takas tutarı içerisinden tahsil edilir. İlgili tutarlarda değişiklik olması durumunda internet sayfamızda güncellenmektedir.</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3953,7 +3701,6 @@
           <t>0.084%</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr">
         <is>
           <t>0.0105%</t>
@@ -3964,7 +3711,6 @@
           <t>Hesap açılışında komisyon oranı sabit 0,084% (onbinde 8,4) olarak atanmaktadır. Oranlar işlem başına olup, BSMV dahil değildir. Sözleşmelerde belirtildiği üzere yapılan her işlemde (alım/satım), kurum azami BSMV hariç binde 1,05 oranında komisyon tahsilatı yapma hakkına sahiptir. BSMV oranı işlemden kesilen komisyonun yüzde 5’idir.</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -3987,7 +3733,6 @@
           <t>0.001%</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
           <t>0.001%</t>
@@ -3998,7 +3743,6 @@
           <t>BSMV hariç.</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4021,14 +3765,11 @@
           <t>0.01%</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr"/>
-      <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
           <t>İşlem Piyasa Değeri</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4046,15 +3787,11 @@
           <t>139.21TL</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr"/>
-      <c r="D117" t="inlineStr"/>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>İşlem sayısı</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4072,15 +3809,11 @@
           <t>1.39TL</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr"/>
-      <c r="D118" t="inlineStr"/>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>İşlem sayısı</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4098,15 +3831,11 @@
           <t>17.75TL</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>Açılan hesap başına</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4124,7 +3853,6 @@
           <t>13.05TL</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
           <t>25.78TL</t>
@@ -4140,7 +3868,6 @@
           <t>Talimat sayısı</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4158,7 +3885,6 @@
           <t>1.38TL</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr">
         <is>
           <t>6.90TL</t>
@@ -4174,7 +3900,6 @@
           <t>Talimat sayısı</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4192,19 +3917,16 @@
           <t>160.00TL</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr">
         <is>
           <t>180.00TL</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
           <t>Asgari Tutar; yurt içi yerleşik ekran ücretlerini, Azami Tutar ise yurt dışı yerleşik (KKTC dahil) ekran ücretlerini göstermektedir. Ücretler aylık olarak tahsil edilmektedir.</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4252,19 +3974,16 @@
           <t>0TL</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
           <t>300.00TL</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>Asgari Tutar; yurt içi yerleşik ekran ücretlerini, Azami Tutar ise yurt dışı yerleşik (KKTC dahil) ekran ücretlerini göstermektedir. Ücretler aylık olarak tahsil edilmektedir.</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4282,19 +4001,16 @@
           <t>600.00TL</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
           <t>945.00TL</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
           <t>Asgari Tutar; yurt içi yerleşik ekran ücretlerini, Azami Tutar ise yurt dışı yerleşik (KKTC dahil) ekran ücretlerini göstermektedir. Ücretler aylık olarak tahsil edilmektedir.</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4312,19 +4028,16 @@
           <t>980.00TL</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
           <t>1665.00TL</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
           <t>Asgari Tutar; yurt içi yerleşik ekran ücretlerini, Azami Tutar ise yurt dışı yerleşik (KKTC dahil) ekran ücretlerini göstermektedir. Ücretler aylık olarak tahsil edilmektedir.</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4342,19 +4055,16 @@
           <t>1300.00TL</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
           <t>1980.00TL</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
           <t>Asgari Tutar; yurt içi yerleşik ekran ücretlerini, Azami Tutar ise yurt dışı yerleşik (KKTC dahil) ekran ücretlerini göstermektedir. Ücretler aylık olarak tahsil edilmektedir.</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr">
         <is>
           <t>31.07.2026</t>
@@ -4372,19 +4082,16 @@
           <t>540.00TL</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr">
         <is>
           <t>900.00TL</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
         <is>
           <t>Asgari Tutar; yurt içi yerleşik ekran ücretlerini, Azami Tutar ise yurt dışı yerleşik (KKTC dahil) ekran ücretlerini göstermektedir. Ücretler aylık olarak tahsil edilmektedir.</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
           <t>31.07.2026</t>

</xml_diff>